<commit_message>
Update vault (2026-08-26 11:20 IST)
</commit_message>
<xml_diff>
--- a/sem_3/assignments/SDA/OnBoardingForm_AdityaMishra_Lab5.xlsx
+++ b/sem_3/assignments/SDA/OnBoardingForm_AdityaMishra_Lab5.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aditya\mainframe\vault\sem_3\assignments\SDA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{568D33FB-2717-461A-A7A7-8439BE5C0A28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD3EC45D-C3C8-44DA-B3A2-7A23A54DDE41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CE01787A-09D6-42B8-8A68-1189D89147A4}"/>
   </bookViews>
   <sheets>
     <sheet name="Onbording Form" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
-    <sheet name="test_log" sheetId="2" r:id="rId3"/>
+    <sheet name="test_log" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="47">
   <si>
     <t>Emp ID</t>
   </si>
@@ -127,9 +126,6 @@
     <t>Warning</t>
   </si>
   <si>
-    <t>logi</t>
-  </si>
-  <si>
     <t>EMP001</t>
   </si>
   <si>
@@ -148,40 +144,22 @@
     <t>Finance</t>
   </si>
   <si>
-    <t>riya.mehta@gmail</t>
-  </si>
-  <si>
     <t>EMP003</t>
   </si>
   <si>
     <t>Karan Patel</t>
   </si>
   <si>
-    <t>karan.patel@company.com</t>
-  </si>
-  <si>
     <t>EMP004</t>
   </si>
   <si>
     <t>Neha Shah</t>
   </si>
   <si>
-    <t>finanace</t>
-  </si>
-  <si>
-    <t>31-Feb-2019</t>
-  </si>
-  <si>
-    <t>neha.shahcompany.com</t>
-  </si>
-  <si>
     <t>EMP005</t>
   </si>
   <si>
     <t>Aditya Rao</t>
-  </si>
-  <si>
-    <t>aditya.rao@company.com</t>
   </si>
   <si>
     <t>riya.mehta@gmail.com</t>
@@ -679,10 +657,10 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>18</v>
@@ -697,7 +675,7 @@
         <v>4</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H3" s="4">
         <v>92</v>
@@ -705,13 +683,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="6" t="s">
         <v>33</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>34</v>
       </c>
       <c r="D4" s="7">
         <v>45007</v>
@@ -723,7 +701,7 @@
         <v>5</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="H4" s="4">
         <v>88</v>
@@ -731,13 +709,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D5" s="7">
         <v>45818</v>
@@ -749,7 +727,7 @@
         <v>3</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="H5" s="4">
         <v>95</v>
@@ -757,13 +735,13 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="D6" s="7">
         <v>44791</v>
@@ -775,7 +753,7 @@
         <v>4</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="H6" s="4">
         <v>90</v>
@@ -783,13 +761,13 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="D7" s="7">
         <v>44444</v>
@@ -801,7 +779,7 @@
         <v>3</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="H7" s="4">
         <v>86</v>
@@ -872,11 +850,11 @@
       <formula1>3</formula1>
       <formula2>40</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G8:G20" xr:uid="{40180297-69B8-4290-B6CE-0C86BBAE17AE}">
-      <formula1>AND(ISNUMBER(SEARCH("@",G3)),ISNUMBER(SEARCH(".",G3)),COUNTIF($G$2:$G$20,G3)=1)</formula1>
-    </dataValidation>
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A8:A20" xr:uid="{F043F0C5-1241-4D14-97A9-87E52641ED05}">
       <formula1>AND(LEFT(A8,3)="EMP",LEN(A8)=6)</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G20" xr:uid="{AEE967B2-F53A-4467-9799-09A9B7D88A3B}">
+      <formula1>AND(ISNUMBER(SEARCH("@",G2)),ISNUMBER(SEARCH(".",G2)),LEN(G2)-LEN(SUBSTITUTE(G2,"@",""))=1,LEFT(G2,1)&lt;&gt;"@",RIGHT(G2,1)&lt;&gt;"@",ISNUMBER(SEARCH(".",MID(G2,SEARCH("@",G2)+1,999))),COUNTIF($G$2:$G$1048574,G2)=1)</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -892,186 +870,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{33AF03C6-659E-4ADC-A221-2F7E606C429D}">
-  <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="7">
-        <v>45306</v>
-      </c>
-      <c r="E2" s="4">
-        <v>45000</v>
-      </c>
-      <c r="F2" s="4">
-        <v>4</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="H2" s="4">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D3" s="7">
-        <v>43181</v>
-      </c>
-      <c r="E3" s="4">
-        <v>52000</v>
-      </c>
-      <c r="F3" s="4">
-        <v>5</v>
-      </c>
-      <c r="G3" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="H3" s="4">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="60" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="7">
-        <v>45818</v>
-      </c>
-      <c r="E4" s="4">
-        <v>-25000</v>
-      </c>
-      <c r="F4" s="4">
-        <v>3</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="4">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="E5" s="4">
-        <v>68000</v>
-      </c>
-      <c r="F5" s="4">
-        <v>6</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" s="4">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D6" s="7">
-        <v>42983</v>
-      </c>
-      <c r="E6" s="4">
-        <v>-15000</v>
-      </c>
-      <c r="F6" s="4">
-        <v>2</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="H6" s="4">
-        <v>-10</v>
-      </c>
-    </row>
-  </sheetData>
-  <hyperlinks>
-    <hyperlink ref="G2" r:id="rId1" display="mailto:aarav.sharma@gmail.com" xr:uid="{486FF36F-BEC2-4851-BB7A-E417E203D34C}"/>
-    <hyperlink ref="G4" r:id="rId2" display="mailto:karan.patel@company.com" xr:uid="{6FD9B3FE-BFA2-40B0-A0F9-23943BC572A5}"/>
-    <hyperlink ref="G6" r:id="rId3" display="mailto:aditya.rao@company.com" xr:uid="{48391A9F-493B-47D9-8C55-4855C00E2D66}"/>
-  </hyperlinks>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C027673-1432-4002-9703-29340D6AC700}">
   <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1302,7 +1100,7 @@
         <v>21</v>
       </c>
       <c r="C21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>